<commit_message>
List the 47 checkpoint genes in Supplementary Table S2e
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/supplementary_tables/Supplementary_Table_S2.xlsx
+++ b/supplementary_tables/Supplementary_Table_S2.xlsx
@@ -10,12 +10,13 @@
     <sheet name="S2b_corpus_keywords" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="S2c_modules" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="S2d_gene_sets" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="S2e_checkpoint_genes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="207">
   <si>
     <t xml:space="preserve">Supplementary Table S2a. PubMed queries (searched 15 October 2026), hits and records retrieved.</t>
   </si>
@@ -489,6 +490,153 @@
   </si>
   <si>
     <t xml:space="preserve">GOBP_ANOIKIS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supplementary Table S2e. Immune checkpoint genes tested in the immune-checkpoint module (M13; n = 47).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gene</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDO1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAG3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTLA4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNFRSF9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PDCD1LG2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TIGIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNFSF9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICOSLG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KIR3DL1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD86</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PDCD1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAIR1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNFRSF8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNFSF15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNFRSF14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDO2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD276</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNFRSF4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNFSF14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HHLA2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD244</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD274</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HAVCR2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BTLA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LGALS9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMIGD2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNFRSF25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD40LG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADORA2A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VTCN1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD160</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNFSF18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNFRSF18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BTNL2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VSIR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD200R1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNFSF4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRP1</t>
   </si>
 </sst>
 </file>
@@ -1812,4 +1960,260 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>206</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>